<commit_message>
Update MLB hitter fantasy scores 2026-07-12 (2026-07-11 09:56 PM)
</commit_message>
<xml_diff>
--- a/PRIZEPICKS_HITTER_AI_V3_TOP30_2026_07_12.xlsx
+++ b/PRIZEPICKS_HITTER_AI_V3_TOP30_2026_07_12.xlsx
@@ -1989,13 +1989,13 @@
         <v>1.03</v>
       </c>
       <c r="BC4" s="3" t="n">
-        <v>81.3</v>
+        <v>81.8</v>
       </c>
       <c r="BD4" s="3" t="n">
-        <v>7.9</v>
+        <v>6.2</v>
       </c>
       <c r="BE4" s="3" t="n">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="BF4" s="3" t="n">
         <v>6</v>
@@ -2331,13 +2331,13 @@
         <v>1.03</v>
       </c>
       <c r="BC5" s="3" t="n">
-        <v>85.5</v>
+        <v>85.2</v>
       </c>
       <c r="BD5" s="3" t="n">
-        <v>8.5</v>
+        <v>8.4</v>
       </c>
       <c r="BE5" s="3" t="n">
-        <v>88</v>
+        <v>99</v>
       </c>
       <c r="BF5" s="3" t="n">
         <v>8</v>
@@ -2673,13 +2673,13 @@
         <v>1.01</v>
       </c>
       <c r="BC6" s="3" t="n">
-        <v>72.7</v>
+        <v>72.3</v>
       </c>
       <c r="BD6" s="3" t="n">
         <v>12.6</v>
       </c>
       <c r="BE6" s="3" t="n">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="BF6" s="3" t="n">
         <v>2</v>
@@ -3015,13 +3015,13 @@
         <v>1.01</v>
       </c>
       <c r="BC7" s="3" t="n">
-        <v>72.7</v>
+        <v>72.3</v>
       </c>
       <c r="BD7" s="3" t="n">
         <v>12.6</v>
       </c>
       <c r="BE7" s="3" t="n">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="BF7" s="3" t="n">
         <v>2</v>
@@ -3357,13 +3357,13 @@
         <v>1.01</v>
       </c>
       <c r="BC8" s="3" t="n">
-        <v>72.7</v>
+        <v>72.3</v>
       </c>
       <c r="BD8" s="3" t="n">
         <v>12.6</v>
       </c>
       <c r="BE8" s="3" t="n">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="BF8" s="3" t="n">
         <v>2</v>
@@ -4033,13 +4033,13 @@
         <v>1.03</v>
       </c>
       <c r="BC10" s="3" t="n">
-        <v>85.5</v>
+        <v>85.2</v>
       </c>
       <c r="BD10" s="3" t="n">
-        <v>8.5</v>
+        <v>8.4</v>
       </c>
       <c r="BE10" s="3" t="n">
-        <v>88</v>
+        <v>99</v>
       </c>
       <c r="BF10" s="3" t="n">
         <v>8</v>
@@ -4709,13 +4709,13 @@
         <v>1.03</v>
       </c>
       <c r="BC12" s="3" t="n">
-        <v>81.8</v>
+        <v>81.40000000000001</v>
       </c>
       <c r="BD12" s="3" t="n">
-        <v>3</v>
+        <v>2.7</v>
       </c>
       <c r="BE12" s="3" t="n">
-        <v>63</v>
+        <v>55</v>
       </c>
       <c r="BF12" s="3" t="n">
         <v>1</v>
@@ -5051,13 +5051,13 @@
         <v>1.03</v>
       </c>
       <c r="BC13" s="3" t="n">
-        <v>86.2</v>
+        <v>86</v>
       </c>
       <c r="BD13" s="3" t="n">
-        <v>8.5</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="BE13" s="3" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="BF13" s="3" t="n">
         <v>0</v>
@@ -5393,13 +5393,13 @@
         <v>1.03</v>
       </c>
       <c r="BC14" s="3" t="n">
-        <v>81.3</v>
+        <v>81.8</v>
       </c>
       <c r="BD14" s="3" t="n">
-        <v>7.9</v>
+        <v>6.2</v>
       </c>
       <c r="BE14" s="3" t="n">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="BF14" s="3" t="n">
         <v>6</v>
@@ -6403,13 +6403,13 @@
         <v>1.01</v>
       </c>
       <c r="BC17" s="3" t="n">
-        <v>72.7</v>
+        <v>72.3</v>
       </c>
       <c r="BD17" s="3" t="n">
         <v>12.6</v>
       </c>
       <c r="BE17" s="3" t="n">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="BF17" s="3" t="n">
         <v>2</v>
@@ -6745,13 +6745,13 @@
         <v>1.03</v>
       </c>
       <c r="BC18" s="3" t="n">
-        <v>85.3</v>
+        <v>85.2</v>
       </c>
       <c r="BD18" s="3" t="n">
-        <v>7.2</v>
+        <v>7.5</v>
       </c>
       <c r="BE18" s="3" t="n">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="BF18" s="3" t="n">
         <v>4</v>
@@ -7087,13 +7087,13 @@
         <v>1</v>
       </c>
       <c r="BC19" s="3" t="n">
-        <v>78.7</v>
+        <v>78.09999999999999</v>
       </c>
       <c r="BD19" s="3" t="n">
-        <v>7.9</v>
+        <v>8.1</v>
       </c>
       <c r="BE19" s="3" t="n">
-        <v>250</v>
+        <v>264</v>
       </c>
       <c r="BF19" s="3" t="n">
         <v>2</v>
@@ -7429,13 +7429,13 @@
         <v>1.03</v>
       </c>
       <c r="BC20" s="3" t="n">
-        <v>85.5</v>
+        <v>85.2</v>
       </c>
       <c r="BD20" s="3" t="n">
-        <v>8.5</v>
+        <v>8.4</v>
       </c>
       <c r="BE20" s="3" t="n">
-        <v>88</v>
+        <v>99</v>
       </c>
       <c r="BF20" s="3" t="n">
         <v>8</v>
@@ -7771,13 +7771,13 @@
         <v>1.03</v>
       </c>
       <c r="BC21" s="3" t="n">
-        <v>81.3</v>
+        <v>81.8</v>
       </c>
       <c r="BD21" s="3" t="n">
-        <v>7.9</v>
+        <v>6.2</v>
       </c>
       <c r="BE21" s="3" t="n">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="BF21" s="3" t="n">
         <v>6</v>
@@ -8781,13 +8781,13 @@
         <v>1.03</v>
       </c>
       <c r="BC24" s="3" t="n">
-        <v>81.3</v>
+        <v>81.8</v>
       </c>
       <c r="BD24" s="3" t="n">
-        <v>7.9</v>
+        <v>6.2</v>
       </c>
       <c r="BE24" s="3" t="n">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="BF24" s="3" t="n">
         <v>6</v>
@@ -9457,13 +9457,13 @@
         <v>1.01</v>
       </c>
       <c r="BC26" s="3" t="n">
-        <v>72.7</v>
+        <v>72.3</v>
       </c>
       <c r="BD26" s="3" t="n">
         <v>12.6</v>
       </c>
       <c r="BE26" s="3" t="n">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="BF26" s="3" t="n">
         <v>2</v>
@@ -9799,13 +9799,13 @@
         <v>1.01</v>
       </c>
       <c r="BC27" s="3" t="n">
-        <v>72.7</v>
+        <v>72.3</v>
       </c>
       <c r="BD27" s="3" t="n">
         <v>12.6</v>
       </c>
       <c r="BE27" s="3" t="n">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="BF27" s="3" t="n">
         <v>2</v>
@@ -10475,13 +10475,13 @@
         <v>1.01</v>
       </c>
       <c r="BC29" s="3" t="n">
-        <v>72.7</v>
+        <v>72.3</v>
       </c>
       <c r="BD29" s="3" t="n">
         <v>12.6</v>
       </c>
       <c r="BE29" s="3" t="n">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="BF29" s="3" t="n">
         <v>2</v>
@@ -11151,13 +11151,13 @@
         <v>1.055</v>
       </c>
       <c r="BC31" s="3" t="n">
-        <v>91.90000000000001</v>
+        <v>91.7</v>
       </c>
       <c r="BD31" s="3" t="n">
-        <v>8.800000000000001</v>
+        <v>8.1</v>
       </c>
       <c r="BE31" s="3" t="n">
-        <v>216</v>
+        <v>233</v>
       </c>
       <c r="BF31" s="3" t="n">
         <v>0</v>

</xml_diff>